<commit_message>
Master monitor and PRD record what is built
New tab "Built - Aug 11" in the master monitor: 18 built items in five
groups, each with what was wrong, what is built and which instruction it
came from, plus the one Performance item left open on purpose. A pointer
row on the SUMMARY tab. The 44 existing status rows are untouched - none
of them is what this work covered.

PRD gains an Amendments row pointing at the tab; same-day changelog row;
dated snapshots of all three workbooks.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-PRD-v1.1-2026-07-01.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-PRD-v1.1-2026-07-01.xlsx
@@ -875,7 +875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -1085,6 +1085,28 @@
       <c r="D9" s="31" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-11: "where are we getting data or assumptions for monte carlo simulation?" → fix the weak assumption, explain it to a non-finance reader, and record it in the master PRD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>Build status — what is built vs what the documents ask for</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>The 2026-08-11 build is recorded in the master monitor (docs/FCC-core-55-70/build-analysis-july24.xlsx, tab "Built — Aug 11"): 18 items covering the Net worth Quiet-Instrument rebuild, the connection-honesty fixes, the classification chain (cash means cash; the leftover is cash; a deposit lands in cash), the retirement plan (the verdict speaks below 80%, the three-questions screen, what counts toward retirement, measured volatility, the plain-English method), and the account-detail / Performance handoff. Each row carries what was wrong, what is built, and where the instruction came from. TWO items remain open by the founder's own instruction: a category-detail screen, and the handoff's "/yr" stated-yield treatment for bonds and cash, which is a calculation change rather than UX.</t>
+        </is>
+      </c>
+      <c r="D10" s="31" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-11: "Update master PRD document. Go to master list of what's missing in app versus PRD, and update it listing what already build."</t>
         </is>
       </c>
     </row>

</xml_diff>